<commit_message>
Add new French advisors and portraits, update character data
Added several new French advisor entries and their corresponding portrait files. Updated FRA.txt to include new portrait references and a corps commander for Paul Nord. Modified event traits for Louis Bonaparte. Added a utility Python script for registering advisor and character portraits. Updated FRA_advisor.gfx to register new advisor portraits and renamed Paul Nord's advisor portrait file for consistency.
</commit_message>
<xml_diff>
--- a/WIP/工作簿222.xlsx
+++ b/WIP/工作簿222.xlsx
@@ -513,11 +513,34 @@
       </xdr:spPr>
     </xdr:pic>
   </etc:cellImage>
+  <etc:cellImage>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="ID_F56B23B77059461E90EA9E9FFA24906D" descr="Portrait_FRA_Julia_Bonaparte"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1981200" cy="2667000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+  </etc:cellImage>
 </etc:cellImages>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="57">
   <si>
     <t>法兰西共和国</t>
   </si>
@@ -645,43 +668,46 @@
     <t>洛朗丝·让娜·特雷布</t>
   </si>
   <si>
+    <t>茱莉娅·波拿巴</t>
+  </si>
+  <si>
+    <t>拿破仑六世</t>
+  </si>
+  <si>
+    <t>国民议会</t>
+  </si>
+  <si>
+    <t>联盟选举-总工会胜出</t>
+  </si>
+  <si>
+    <t>联盟选举-共产党胜出</t>
+  </si>
+  <si>
+    <t>中央政治局</t>
+  </si>
+  <si>
+    <t>莫里斯·多列士</t>
+  </si>
+  <si>
+    <t>普鲁士王国</t>
+  </si>
+  <si>
+    <t>国王</t>
+  </si>
+  <si>
+    <t>腓特烈三世</t>
+  </si>
+  <si>
+    <t>古斯塔夫·施特雷泽曼</t>
+  </si>
+  <si>
+    <t>施特雷泽曼病逝</t>
+  </si>
+  <si>
+    <t>国王任命</t>
+  </si>
+  <si>
     <t>路易·波拿巴</t>
-  </si>
-  <si>
-    <t>拿破仑六世</t>
-  </si>
-  <si>
-    <t>国民议会</t>
-  </si>
-  <si>
-    <t>联盟选举-总工会胜出</t>
-  </si>
-  <si>
-    <t>联盟选举-共产党胜出</t>
-  </si>
-  <si>
-    <t>中央政治局</t>
-  </si>
-  <si>
-    <t>莫里斯·多列士</t>
-  </si>
-  <si>
-    <t>普鲁士王国</t>
-  </si>
-  <si>
-    <t>国王</t>
-  </si>
-  <si>
-    <t>腓特烈三世</t>
-  </si>
-  <si>
-    <t>古斯塔夫·施特雷泽曼</t>
-  </si>
-  <si>
-    <t>施特雷泽曼病逝</t>
-  </si>
-  <si>
-    <t>国王任命</t>
   </si>
   <si>
     <t>最后的晚餐</t>
@@ -2396,8 +2422,8 @@
         <v>=DISPIMG("ID_BBD8047041E6437CA612318FDBCECE2B",1)</v>
       </c>
       <c r="U27" s="7" t="str">
-        <f>_xlfn.DISPIMG("ID_D01F21D8B2764EB7AEC65BF3E9C1B7DF",1)</f>
-        <v>=DISPIMG("ID_D01F21D8B2764EB7AEC65BF3E9C1B7DF",1)</v>
+        <f>_xlfn.DISPIMG("ID_F56B23B77059461E90EA9E9FFA24906D",1)</f>
+        <v>=DISPIMG("ID_F56B23B77059461E90EA9E9FFA24906D",1)</v>
       </c>
       <c r="V27"/>
       <c r="Y27" s="2" t="str">
@@ -3171,7 +3197,7 @@
         <v>41</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="N28"/>
       <c r="Q28" s="5" t="s">
@@ -3345,7 +3371,7 @@
   <sheetData>
     <row r="3" spans="7:7">
       <c r="G3" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="7:7">

</xml_diff>

<commit_message>
Add shared Reich focus and update localisation
Introduced HV_reich_shared.txt with new shared and joint focuses for Reich, referenced in Prussia and Austria focus trees. Added new Chinese localisation entries for '天堂之梦' and related country descriptions.
</commit_message>
<xml_diff>
--- a/WIP/工作簿222.xlsx
+++ b/WIP/工作簿222.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="17655"/>
+    <workbookView windowWidth="27885" windowHeight="12375" firstSheet="1" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="法国" sheetId="1" r:id="rId1"/>
@@ -609,7 +609,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="86">
   <si>
     <t>法兰西共和国</t>
   </si>
@@ -800,7 +800,73 @@
     <t>库尔特·冯·施莱歇尔</t>
   </si>
   <si>
-    <t>在神罗的最后一日</t>
+    <t>前路漫漫……</t>
+  </si>
+  <si>
+    <t>（施特雷泽曼病逝）</t>
+  </si>
+  <si>
+    <t>……终有竟时</t>
+  </si>
+  <si>
+    <t>事件“在柏林的最后一日”</t>
+  </si>
+  <si>
+    <t>将军</t>
+  </si>
+  <si>
+    <t>&lt;-!-&gt;</t>
+  </si>
+  <si>
+    <t>最后机会</t>
+  </si>
+  <si>
+    <t>一线生机</t>
+  </si>
+  <si>
+    <t>广撒情报网</t>
+  </si>
+  <si>
+    <t>争取皇帝支持</t>
+  </si>
+  <si>
+    <t>民族浪潮</t>
+  </si>
+  <si>
+    <t>阴影之触</t>
+  </si>
+  <si>
+    <t>承诺安全保障</t>
+  </si>
+  <si>
+    <t>和平外交</t>
+  </si>
+  <si>
+    <t>潜伏的支持者们</t>
+  </si>
+  <si>
+    <t>抛出橄榄枝</t>
+  </si>
+  <si>
+    <t>统一的帝国铁路网络</t>
+  </si>
+  <si>
+    <t>巩固基本盘</t>
+  </si>
+  <si>
+    <t>重新商讨各邦国的地位</t>
+  </si>
+  <si>
+    <t>弃车保帅</t>
+  </si>
+  <si>
+    <t>工业支援</t>
+  </si>
+  <si>
+    <t>南德意志经济合作同盟</t>
+  </si>
+  <si>
+    <t>沉默的议案</t>
   </si>
 </sst>
 </file>
@@ -2018,13 +2084,13 @@
     <col min="9" max="16384" width="22.775" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="7" spans="15:16">
+    <row r="7" spans="13:30">
       <c r="O7" s="3" t="s">
         <v>0</v>
       </c>
       <c r="P7" s="3"/>
     </row>
-    <row r="8" spans="15:16">
+    <row r="8" spans="13:30">
       <c r="O8" s="4" t="s">
         <v>1</v>
       </c>
@@ -2032,7 +2098,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="164.95" spans="15:16">
+    <row r="9" ht="164.95" spans="13:30">
       <c r="O9" s="2" t="str">
         <f>_xlfn.DISPIMG("ID_493F53998CA04DB19D50C21913B05A8E",1)</f>
         <v>=DISPIMG("ID_493F53998CA04DB19D50C21913B05A8E",1)</v>
@@ -2042,7 +2108,7 @@
         <v>=DISPIMG("ID_B518E24FC4B44BDD8CE2A00C429D6F95",1)</v>
       </c>
     </row>
-    <row r="10" spans="15:16">
+    <row r="10" spans="13:30">
       <c r="O10" s="5" t="s">
         <v>3</v>
       </c>
@@ -2050,17 +2116,17 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="15:15">
+    <row r="11" spans="13:30">
       <c r="O11" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="15:15">
+    <row r="12" spans="13:30">
       <c r="O12" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="13:29">
+    <row r="13" spans="13:30">
       <c r="M13" s="2" t="s">
         <v>6</v>
       </c>
@@ -2113,7 +2179,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="13:29">
+    <row r="14" spans="13:30">
       <c r="M14" s="2" t="s">
         <v>5</v>
       </c>
@@ -2184,7 +2250,7 @@
       </c>
       <c r="AD16" s="3"/>
     </row>
-    <row r="17" spans="13:30">
+    <row r="17" spans="5:30">
       <c r="M17" s="4" t="s">
         <v>1</v>
       </c>
@@ -2216,7 +2282,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" ht="165" customHeight="1" spans="13:30">
+    <row r="18" ht="165" customHeight="1" spans="5:30">
       <c r="M18" s="2" t="str">
         <f>_xlfn.DISPIMG("ID_9B5E25B467354840860B770A994B94D9",1)</f>
         <v>=DISPIMG("ID_9B5E25B467354840860B770A994B94D9",1)</v>
@@ -2258,7 +2324,7 @@
         <v>=DISPIMG("ID_B518E24FC4B44BDD8CE2A00C429D6F95",1)</v>
       </c>
     </row>
-    <row r="19" spans="13:30">
+    <row r="19" spans="5:30">
       <c r="M19" s="5" t="s">
         <v>12</v>
       </c>
@@ -2290,7 +2356,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="13:29">
+    <row r="20" spans="5:30">
       <c r="M20" s="2" t="s">
         <v>5</v>
       </c>
@@ -2307,7 +2373,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="13:29">
+    <row r="21" spans="5:30">
       <c r="M21" s="2" t="s">
         <v>5</v>
       </c>
@@ -2324,7 +2390,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="9:29">
+    <row r="22" spans="5:30">
       <c r="I22" s="2" t="s">
         <v>6</v>
       </c>
@@ -2362,7 +2428,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="9:29">
+    <row r="23" spans="5:30">
       <c r="I23" s="2" t="s">
         <v>5</v>
       </c>
@@ -2384,7 +2450,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="9:30">
+    <row r="24" spans="5:30">
       <c r="I24" s="2" t="s">
         <v>5</v>
       </c>
@@ -2418,7 +2484,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="9:30">
+    <row r="25" spans="5:30">
       <c r="I25" s="3" t="s">
         <v>21</v>
       </c>
@@ -2443,7 +2509,7 @@
       </c>
       <c r="AD25" s="3"/>
     </row>
-    <row r="26" spans="9:30">
+    <row r="26" spans="5:30">
       <c r="I26" s="4" t="s">
         <v>25</v>
       </c>
@@ -2482,7 +2548,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="27" ht="165" customHeight="1" spans="9:30">
+    <row r="27" ht="165" customHeight="1" spans="5:30">
       <c r="I27" s="2" t="str">
         <f>_xlfn.DISPIMG("ID_A30A5F3F6621414284AC160534B321A3",1)</f>
         <v>=DISPIMG("ID_A30A5F3F6621414284AC160534B321A3",1)</v>
@@ -2533,7 +2599,7 @@
         <v>=DISPIMG("ID_5DB37D32B60343BBB2A8FA65F262AFD8",1)</v>
       </c>
     </row>
-    <row r="28" spans="9:30">
+    <row r="28" spans="5:30">
       <c r="I28" s="5" t="s">
         <v>35</v>
       </c>
@@ -2573,17 +2639,17 @@
         <v>44</v>
       </c>
     </row>
-    <row r="29" spans="9:9">
+    <row r="29" spans="5:30">
       <c r="I29" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="9:9">
+    <row r="30" spans="5:30">
       <c r="I30" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="5:18">
+    <row r="31" spans="5:30">
       <c r="E31" s="2" t="s">
         <v>6</v>
       </c>
@@ -2609,7 +2675,7 @@
       <c r="Q31"/>
       <c r="R31"/>
     </row>
-    <row r="32" spans="5:18">
+    <row r="32" spans="5:30">
       <c r="E32" s="2" t="s">
         <v>5</v>
       </c>
@@ -2753,13 +2819,13 @@
     <col min="1" max="16384" width="22.775" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="7" spans="7:8">
+    <row r="7" spans="5:22">
       <c r="G7" s="3" t="s">
         <v>49</v>
       </c>
       <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="7:8">
+    <row r="8" spans="5:22">
       <c r="G8" s="4" t="s">
         <v>50</v>
       </c>
@@ -2767,7 +2833,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" ht="165" spans="7:8">
+    <row r="9" ht="165" spans="5:22">
       <c r="G9" s="2" t="str">
         <f>_xlfn.DISPIMG("ID_8BE45564F174476EB008DF96A41A0EA6",1)</f>
         <v>=DISPIMG("ID_8BE45564F174476EB008DF96A41A0EA6",1)</v>
@@ -2777,7 +2843,7 @@
         <v>=DISPIMG("ID_125BAE01ADED4FB19EAE7E7A165B5877",1)</v>
       </c>
     </row>
-    <row r="10" spans="7:8">
+    <row r="10" spans="5:22">
       <c r="G10" s="5" t="s">
         <v>51</v>
       </c>
@@ -2785,12 +2851,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="7:7">
+    <row r="11" spans="5:22">
       <c r="G11" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="7:9">
+    <row r="12" spans="5:22">
       <c r="G12" s="2" t="s">
         <v>5</v>
       </c>
@@ -2918,7 +2984,7 @@
       <c r="U16"/>
       <c r="V16"/>
     </row>
-    <row r="17" spans="5:22">
+    <row r="17" spans="1:22">
       <c r="E17" s="4" t="s">
         <v>50</v>
       </c>
@@ -2947,7 +3013,7 @@
       <c r="U17"/>
       <c r="V17"/>
     </row>
-    <row r="18" ht="165" customHeight="1" spans="5:22">
+    <row r="18" ht="165" customHeight="1" spans="1:22">
       <c r="E18" s="2" t="str">
         <f>_xlfn.DISPIMG("ID_8BE45564F174476EB008DF96A41A0EA6",1)</f>
         <v>=DISPIMG("ID_8BE45564F174476EB008DF96A41A0EA6",1)</v>
@@ -2984,7 +3050,7 @@
       <c r="U18"/>
       <c r="V18"/>
     </row>
-    <row r="19" spans="5:22">
+    <row r="19" spans="1:22">
       <c r="E19" s="5" t="s">
         <v>51</v>
       </c>
@@ -3013,7 +3079,7 @@
       <c r="U19"/>
       <c r="V19"/>
     </row>
-    <row r="20" spans="5:22">
+    <row r="20" spans="1:22">
       <c r="E20" s="2" t="s">
         <v>5</v>
       </c>
@@ -3030,7 +3096,7 @@
       <c r="U20"/>
       <c r="V20"/>
     </row>
-    <row r="21" spans="5:22">
+    <row r="21" spans="1:22">
       <c r="E21" s="2" t="s">
         <v>5</v>
       </c>
@@ -3208,7 +3274,7 @@
       <c r="U28"/>
       <c r="V28"/>
     </row>
-    <row r="29" spans="1:18">
+    <row r="29" spans="1:22">
       <c r="A29"/>
       <c r="B29"/>
       <c r="C29"/>
@@ -3228,7 +3294,7 @@
       <c r="Q29"/>
       <c r="R29"/>
     </row>
-    <row r="30" spans="1:18">
+    <row r="30" spans="1:22">
       <c r="A30"/>
       <c r="B30"/>
       <c r="C30"/>
@@ -3248,7 +3314,7 @@
       <c r="Q30"/>
       <c r="R30"/>
     </row>
-    <row r="31" spans="1:18">
+    <row r="31" spans="1:22">
       <c r="A31"/>
       <c r="B31"/>
       <c r="C31"/>
@@ -3268,7 +3334,7 @@
       <c r="Q31"/>
       <c r="R31"/>
     </row>
-    <row r="32" spans="1:18">
+    <row r="32" spans="1:22">
       <c r="A32"/>
       <c r="B32"/>
       <c r="C32"/>
@@ -3404,39 +3470,307 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="E3:G6"/>
-  <sheetFormatPr defaultColWidth="20.775" defaultRowHeight="13.5" outlineLevelRow="5" outlineLevelCol="6"/>
+  <dimension ref="C3:R15"/>
+  <sheetFormatPr defaultColWidth="20.775" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="16384" width="20.775" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="7:7">
-      <c r="G3" s="1" t="s">
+    <row r="3" spans="3:18">
+      <c r="K3" s="1" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="4" spans="7:7">
-      <c r="G4" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="5:7">
-      <c r="E5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="5:7">
-      <c r="E6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>5</v>
+      <c r="L3" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="3:18">
+      <c r="K4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="3:18">
+      <c r="H5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="3:18">
+      <c r="H6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="3:18">
+      <c r="H7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8" spans="3:18">
+      <c r="H8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="3:18">
+      <c r="D9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="R9" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="3:18">
+      <c r="D10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="3:18">
+      <c r="D11" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="3:18">
+      <c r="D12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="R12" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="3:18">
+      <c r="C13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="R13" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="3:18">
+      <c r="C14" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N14" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P14" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="R14" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="3:18">
+      <c r="C15" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="P15" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="R15" s="1" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>